<commit_message>
State info: Georgia's Oct 6 order
The excise suspension now runs Sept 29 to Nov 5 (EO 10.06.26.01), the
dyed diesel penalty waiver is a row of its own, Oct 6 to Nov 5, and the
prepaid local price cites the July 1, 2026 bulletin.
</commit_message>
<xml_diff>
--- a/General/State info/State Info.xlsx
+++ b/General/State info/State Info.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F95A05B-FCAD-44E7-80CF-62A9F77A736F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF1492D-5283-4024-A50B-958CF3AA32D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="State" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="202">
   <si>
     <t>State info</t>
   </si>
@@ -237,7 +237,7 @@
     <t>(877) 423-6711</t>
   </si>
   <si>
-    <t>Two sales tax returns, on-road and off-road, both laid out like the ST-3. On-road is gallons by county, two lines per county, and Fulton County splits by rate. State excise suspended Sept 29 to Oct 29, 2026.</t>
+    <t>Two sales tax returns, on-road and off-road, both laid out like the ST-3. On-road is gallons by county, two lines per county, and Fulton County splits by rate. State excise suspended Sept 29 to Nov 5, 2026, and state penalties for dyed diesel on the road waived Oct 6 to Nov 5.</t>
   </si>
   <si>
     <t>https://dor.georgia.gov/find-contact-information-topic</t>
@@ -519,7 +519,7 @@
     <t>State motor fuel excise</t>
   </si>
   <si>
-    <t>Schedules of Receipts and Disbursements. Sept 29 to Oct 29, 2026: report the gallons on both schedules, don't remit the excise.</t>
+    <t>Schedules of Receipts and Disbursements. Sept 29 to Nov 5, 2026: report the gallons on both schedules, don't remit the excise.</t>
   </si>
   <si>
     <t>https://dor.georgia.gov/2026-suspension-georgia-motor-fuel-taxes-faqs</t>
@@ -573,10 +573,7 @@
     <t>State excise, suspended</t>
   </si>
   <si>
-    <t>Governor's order EO 09.28.26.01. Gallons still get reported.</t>
-  </si>
-  <si>
-    <t>https://dor.georgia.gov/mft-2026-02-suspension-georgia-motor-fuel-taxes</t>
+    <t>Governor's order EO 09.28.26.01, extended to Nov 5 by EO 10.06.26.01. Gallons still get reported. Prepaid local tax isn't suspended.</t>
   </si>
   <si>
     <t>Prepaid local sales tax</t>
@@ -585,10 +582,22 @@
     <t>see notes</t>
   </si>
   <si>
-    <t>The local rate times a state-set price per gallon, reset each Jan 1 and July 1 and never over $3.00. $3.00 for gas and diesel as of Sept 2026.</t>
-  </si>
-  <si>
-    <t>https://dor.georgia.gov/prepaid-local-tax-motor-fuel-sales-effective-january-1-2026</t>
+    <t>The local rate times a state-set price per gallon, reset each Jan 1 and July 1 and never over $3.00. $3.00 for gas and diesel from July 1, 2026.</t>
+  </si>
+  <si>
+    <t>https://dor.georgia.gov/prepaid-local-tax-motor-fuel-sales-effective-july-1-2026</t>
+  </si>
+  <si>
+    <t>Dyed diesel, road use</t>
+  </si>
+  <si>
+    <t>State penalties waived</t>
+  </si>
+  <si>
+    <t>EO 10.06.26.01 and Bulletin MFT-2026-04 waive the 48-9-16(e) penalties for dyed fuel on the road. The $100 a month notice penalty in (f) still applies.</t>
+  </si>
+  <si>
+    <t>https://dor.georgia.gov/mft-2026-04-temporary-waiver-state-dyed-fuel-penalties</t>
   </si>
   <si>
     <t>Taxpayer Services, motor fuel</t>
@@ -853,8 +862,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="RatesList" displayName="RatesList" ref="A1:J5">
-  <autoFilter ref="A1:J5" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="RatesList" displayName="RatesList" ref="A1:J6">
+  <autoFilter ref="A1:J6" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="State"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Product"/>
@@ -1335,7 +1344,7 @@
       </c>
       <c r="C12" s="20" t="str">
         <f>IF($A$4="","",IF(INDEX(States!I$2:I$1000,$A$4)="","",INDEX(States!I$2:I$1000,$A$4)))</f>
-        <v>Two sales tax returns, on-road and off-road, both laid out like the ST-3. On-road is gallons by county, two lines per county, and Fulton County splits by rate. State excise suspended Sept 29 to Oct 29, 2026.</v>
+        <v>Two sales tax returns, on-road and off-road, both laid out like the ST-3. On-road is gallons by county, two lines per county, and Fulton County splits by rate. State excise suspended Sept 29 to Nov 5, 2026, and state penalties for dyed diesel on the road waived Oct 6 to Nov 5.</v>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="19"/>
@@ -1363,7 +1372,7 @@
       </c>
       <c r="C14" s="21">
         <f>IF($A$4="","",IF(INDEX(States!K$2:K$1000,$A$4)="","",INDEX(States!K$2:K$1000,$A$4)))</f>
-        <v>46296</v>
+        <v>46305</v>
       </c>
       <c r="D14" s="19"/>
       <c r="E14" s="19"/>
@@ -1505,7 +1514,7 @@
       </c>
       <c r="H20" s="10" t="str">
         <f>IF($A20="","",IF(INDEX(Returns!H$2:H$1000,$A20)="","",INDEX(Returns!H$2:H$1000,$A20)))</f>
-        <v>Schedules of Receipts and Disbursements. Sept 29 to Oct 29, 2026: report the gallons on both schedules, don't remit the excise.</v>
+        <v>Schedules of Receipts and Disbursements. Sept 29 to Nov 5, 2026: report the gallons on both schedules, don't remit the excise.</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
@@ -1906,7 +1915,7 @@
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B38" s="6" t="str">
         <f ca="1">"Current rates ("&amp;SUMPRODUCT(((Rates!$A$2:$A$1000=$C$3)*((Rates!$G$2:$G$1000="")+(Rates!$G$2:$G$1000&gt;=TODAY()))))&amp;")"</f>
-        <v>Current rates (4)</v>
+        <v>Current rates (5)</v>
       </c>
       <c r="C38" s="7"/>
       <c r="D38" s="7"/>
@@ -2033,11 +2042,11 @@
       </c>
       <c r="G42" s="13">
         <f ca="1">IF($A42="","",IF(INDEX(Rates!G$2:G$1000,$A42)="","",INDEX(Rates!G$2:G$1000,$A42)))</f>
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="H42" s="10" t="str">
         <f ca="1">IF($A42="","",IF(INDEX(Rates!H$2:H$1000,$A42)="","",INDEX(Rates!H$2:H$1000,$A42)))</f>
-        <v>Governor's order EO 09.28.26.01. Gallons still get reported.</v>
+        <v>Governor's order EO 09.28.26.01, extended to Nov 5 by EO 10.06.26.01. Gallons still get reported. Prepaid local tax isn't suspended.</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
@@ -2071,21 +2080,21 @@
       </c>
       <c r="H43" s="10" t="str">
         <f ca="1">IF($A43="","",IF(INDEX(Rates!H$2:H$1000,$A43)="","",INDEX(Rates!H$2:H$1000,$A43)))</f>
-        <v>The local rate times a state-set price per gallon, reset each Jan 1 and July 1 and never over $3.00. $3.00 for gas and diesel as of Sept 2026.</v>
+        <v>The local rate times a state-set price per gallon, reset each Jan 1 and July 1 and never over $3.00. $3.00 for gas and diesel from July 1, 2026.</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" t="str">
+      <c r="A44">
         <f ca="1">IFERROR(_xlfn.AGGREGATE(15,6,(ROW(Rates!$A$2:$A$1000)-1)/((Rates!$A$2:$A$1000=$C$3)*((Rates!$G$2:$G$1000="")+(Rates!$G$2:$G$1000&gt;=TODAY()))),5),"")</f>
-        <v/>
+        <v>5</v>
       </c>
       <c r="B44" s="11" t="str">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!B$2:B$1000,$A44)="","",INDEX(Rates!B$2:B$1000,$A44)))</f>
-        <v/>
+        <v>Dyed diesel, road use</v>
       </c>
       <c r="C44" s="10" t="str">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!C$2:C$1000,$A44)="","",INDEX(Rates!C$2:C$1000,$A44)))</f>
-        <v/>
+        <v>State penalties waived</v>
       </c>
       <c r="D44" s="11" t="str">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!D$2:D$1000,$A44)="","",INDEX(Rates!D$2:D$1000,$A44)))</f>
@@ -2093,19 +2102,19 @@
       </c>
       <c r="E44" s="10" t="str">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!E$2:E$1000,$A44)="","",INDEX(Rates!E$2:E$1000,$A44)))</f>
-        <v/>
-      </c>
-      <c r="F44" s="13" t="str">
+        <v>see notes</v>
+      </c>
+      <c r="F44" s="13">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!F$2:F$1000,$A44)="","",INDEX(Rates!F$2:F$1000,$A44)))</f>
-        <v/>
-      </c>
-      <c r="G44" s="13" t="str">
+        <v>46301</v>
+      </c>
+      <c r="G44" s="13">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!G$2:G$1000,$A44)="","",INDEX(Rates!G$2:G$1000,$A44)))</f>
-        <v/>
+        <v>46331</v>
       </c>
       <c r="H44" s="10" t="str">
         <f ca="1">IF($A44="","",IF(INDEX(Rates!H$2:H$1000,$A44)="","",INDEX(Rates!H$2:H$1000,$A44)))</f>
-        <v/>
+        <v>EO 10.06.26.01 and Bulletin MFT-2026-04 waive the 48-9-16(e) penalties for dyed fuel on the road. The $100 a month notice penalty in (f) still applies.</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
@@ -2825,7 +2834,7 @@
       <c r="J11" s="11"/>
       <c r="K11" s="13"/>
     </row>
-    <row r="12" spans="1:11" ht="51" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>3</v>
       </c>
@@ -2853,7 +2862,7 @@
         <v>66</v>
       </c>
       <c r="K12" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -3625,7 +3634,7 @@
         <v>153</v>
       </c>
       <c r="J2" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
@@ -3655,7 +3664,7 @@
         <v>153</v>
       </c>
       <c r="J3" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
@@ -3683,7 +3692,7 @@
         <v>160</v>
       </c>
       <c r="J4" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
@@ -3713,7 +3722,7 @@
         <v>167</v>
       </c>
       <c r="J5" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
   </sheetData>
@@ -3809,7 +3818,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -3880,7 +3889,7 @@
         <v>160</v>
       </c>
       <c r="J2" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
@@ -3908,10 +3917,10 @@
         <v>160</v>
       </c>
       <c r="J3" s="13">
-        <v>46296</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+        <v>46305</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>3</v>
       </c>
@@ -3931,16 +3940,16 @@
         <v>46294</v>
       </c>
       <c r="G4" s="13">
-        <v>46324</v>
+        <v>46331</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>177</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="J4" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
@@ -3951,22 +3960,52 @@
         <v>175</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
       <c r="H5" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="I5" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="J5" s="13">
+        <v>46305</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="J5" s="13">
-        <v>46296</v>
+      <c r="C6" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="F6" s="13">
+        <v>46301</v>
+      </c>
+      <c r="G6" s="13">
+        <v>46331</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="J6" s="13">
+        <v>46305</v>
       </c>
     </row>
   </sheetData>
@@ -3980,10 +4019,11 @@
     <hyperlink ref="I3" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
     <hyperlink ref="I4" r:id="rId3" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
     <hyperlink ref="I5" r:id="rId4" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
+    <hyperlink ref="I6" r:id="rId5" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4034,23 +4074,23 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>64</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="G2" s="16" t="s">
         <v>66</v>
       </c>
       <c r="H2" s="13">
-        <v>46296</v>
+        <v>46305</v>
       </c>
     </row>
   </sheetData>
@@ -4138,67 +4178,67 @@
   <sheetData>
     <row r="1" spans="2:2" ht="20.25" x14ac:dyDescent="0.25">
       <c r="B1" s="17" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B3" s="10" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="13" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B13" s="10" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B19" s="10" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="21" spans="2:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="10" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="10" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>